<commit_message>
Sync bs_optimization/ outputs, bump REPORT_DATE to 2026-06-30
REPORT_DATE in anchor_eve_exact.py and swap_ladder.py was still 2024-12-31,
stale against extract_params.REPORT_DATE (2026-06-30) elsewhere in the
pipeline. Also refreshes the regenerated xlsx/png run outputs and a
docstring rename reference (bank_report.ipynb -> ALM_report.ipynb).

Committing this now so bs_optimization/'s full current state is captured
before splitting its history into its own repo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bs_optimization/output/optimal_hedge_swap_input.xlsx
+++ b/bs_optimization/output/optimal_hedge_swap_input.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,11 +524,11 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>45657</v>
+        <v>46203</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IRS_HEDGE_OPT_LADDER_4Y_E017</t>
+          <t>IRS_HEDGE_OPT_LADDER_5Y_E038</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -540,7 +540,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>695883055.4299999</v>
+        <v>999066646.4299999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -548,13 +548,13 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>45138</v>
+        <v>45046</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>46599</v>
+        <v>46873</v>
       </c>
       <c r="I2" t="n">
-        <v>0.06280229714267097</v>
+        <v>0.05503946444344209</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -612,11 +612,11 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>45657</v>
+        <v>46203</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IRS_HEDGE_OPT_LADDER_5Y_E038</t>
+          <t>IRS_HEDGE_OPT_LADDER_3Y_E008</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -628,7 +628,7 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>14481683.15</v>
+        <v>482220832.21</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -636,13 +636,13 @@
         </is>
       </c>
       <c r="G3" s="1" t="n">
-        <v>44500</v>
+        <v>45960</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>46326</v>
+        <v>47056</v>
       </c>
       <c r="I3" t="n">
-        <v>0.01212723446173678</v>
+        <v>0.03750974177885208</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -693,6 +693,94 @@
         </is>
       </c>
       <c r="T3" t="inlineStr">
+        <is>
+          <t>PLN_fwd_curve</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>IRS_HEDGE_OPT_LADDER_6Y_E056</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>IRS</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>933353.5699999999</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>44499</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>46690</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.02510813611717342</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>3M</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ACT/ACT</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>ModifiedFollowing</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>PLN_ASK_3M</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>3M</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>3M</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>ACT/365</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>ModifiedFollowing</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>PLN_disc_curve</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
         <is>
           <t>PLN_fwd_curve</t>
         </is>

</xml_diff>